<commit_message>
Se actualizan los scripts de limpieza de datos
</commit_message>
<xml_diff>
--- a/documentos/DIVIPOLA_Departamentos.xlsx
+++ b/documentos/DIVIPOLA_Departamentos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MAURICIO\DIVIPOLA\ENTREGAS\TRIMESTRE I\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\data_analysis\Portafolio\Inkadata\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3D9383-0CEC-41C4-AFDB-CAF747A252A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C7DB5C5-2E67-4AF4-898D-2D4D9CF7471B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28692" yWindow="-108" windowWidth="15576" windowHeight="11016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Departamentos" sheetId="2" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
@@ -117,9 +117,6 @@
     <t>Departamentos</t>
   </si>
   <si>
-    <t>Código</t>
-  </si>
-  <si>
     <t>Nombre</t>
   </si>
   <si>
@@ -549,6 +546,7 @@
         <sz val="8"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t>Nota:</t>
     </r>
@@ -557,6 +555,7 @@
         <sz val="8"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> En la actualidad el país se compone de 32 departamentos y adicionalmente para fines estadísticos se codifica como departamento el Distrito Capital de Bogotá.</t>
     </r>
@@ -566,13 +565,16 @@
   </si>
   <si>
     <t>Actualizado al 31 de marzo de 2025</t>
+  </si>
+  <si>
+    <t>Codigo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -752,11 +754,20 @@
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1227,7 +1238,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1323,6 +1334,9 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1371,7 +1385,9 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{1985C1B6-26FB-40D1-9E05-2077DE76981B}"/>
+  </tableStyles>
   <colors>
     <mruColors>
       <color rgb="FFB6004B"/>
@@ -1844,14 +1860,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E47"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="56.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" style="24" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" style="24" customWidth="1"/>
-    <col min="5" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="21.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="56.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" style="24" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" style="24" customWidth="1"/>
+    <col min="5" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -1885,7 +1901,7 @@
     </row>
     <row r="6" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="28" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B6" s="28"/>
       <c r="C6" s="28"/>
@@ -1897,7 +1913,7 @@
       <c r="C7" s="28"/>
       <c r="D7" s="28"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="12" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
         <v>0</v>
       </c>
@@ -1905,7 +1921,7 @@
       <c r="C8" s="27"/>
       <c r="D8" s="12"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" ht="12" x14ac:dyDescent="0.2">
       <c r="A9" s="27"/>
       <c r="B9" s="27"/>
       <c r="C9" s="27"/>
@@ -1913,505 +1929,509 @@
     </row>
     <row r="10" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>3</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="D11" s="16" t="s">
         <v>7</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="D12" s="18" t="s">
         <v>11</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="D13" s="16" t="s">
         <v>15</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="D14" s="18" t="s">
         <v>19</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
         <v>15</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="D15" s="16" t="s">
         <v>22</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="D16" s="18" t="s">
         <v>26</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="D17" s="16" t="s">
         <v>30</v>
-      </c>
-      <c r="D17" s="16" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="D18" s="18" t="s">
         <v>34</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="D19" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="D20" s="18" t="s">
         <v>42</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="D21" s="16" t="s">
         <v>46</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="D22" s="18" t="s">
         <v>50</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="D23" s="16" t="s">
         <v>54</v>
-      </c>
-      <c r="D23" s="16" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="C24" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="D24" s="18" t="s">
         <v>58</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="C25" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="D25" s="16" t="s">
         <v>62</v>
-      </c>
-      <c r="D25" s="16" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="C26" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="D26" s="18" t="s">
         <v>66</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="C27" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="19" t="s">
+      <c r="D27" s="16" t="s">
         <v>70</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="C28" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="D28" s="18" t="s">
         <v>74</v>
-      </c>
-      <c r="D28" s="18" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="19" t="s">
+      <c r="D29" s="16" t="s">
         <v>78</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="C30" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="D30" s="18" t="s">
         <v>82</v>
-      </c>
-      <c r="D30" s="18" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="C31" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="D31" s="16" t="s">
         <v>86</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="D32" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="D32" s="18" t="s">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="9" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="9" t="s">
+      <c r="B33" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="C33" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="C33" s="19" t="s">
+      <c r="D33" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="D33" s="16" t="s">
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
+      <c r="B34" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="C34" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="D34" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="D34" s="18" t="s">
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="9" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="9" t="s">
+      <c r="B35" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="C35" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="C35" s="19" t="s">
+      <c r="D35" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="D35" s="16" t="s">
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="8" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="8" t="s">
+      <c r="B36" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="C36" s="17" t="s">
         <v>105</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="D36" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="D36" s="18" t="s">
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="9" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="9" t="s">
+      <c r="B37" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="C37" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="D37" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="D37" s="16" t="s">
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="8" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="8" t="s">
+      <c r="B38" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="C38" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="D38" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="D38" s="18" t="s">
+      <c r="E38" s="1">
+        <f>LEN(B38)</f>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="9" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="9" t="s">
+      <c r="B39" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="C39" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="C39" s="19" t="s">
+      <c r="D39" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="D39" s="16" t="s">
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="8" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="8" t="s">
+      <c r="B40" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="C40" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="D40" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="D40" s="18" t="s">
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="9" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="9" t="s">
+      <c r="B41" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="C41" s="19" t="s">
         <v>125</v>
       </c>
-      <c r="C41" s="19" t="s">
+      <c r="D41" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="D41" s="16" t="s">
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="8" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="8" t="s">
+      <c r="B42" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="C42" s="17" t="s">
         <v>129</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="D42" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="D42" s="18" t="s">
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="10" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="10" t="s">
+      <c r="B43" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="C43" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="C43" s="20" t="s">
+      <c r="D43" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="D43" s="21" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="22"/>
       <c r="D44" s="23"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="34" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B45" s="34"/>
       <c r="C45" s="34"/>
       <c r="D45" s="35"/>
     </row>
-    <row r="46" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="31" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B46" s="32"/>
       <c r="C46" s="32"/>
       <c r="D46" s="33"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" s="29" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B47" s="29"/>
       <c r="C47" s="29"/>
@@ -2439,7 +2459,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2460,15 +2480,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101005130CDF0AED5E24687116040571C2670" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="bbe51c47f34cf99d46406e5cbbd71d04">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="56e6d1e7-6899-430c-9877-67183cfe1730" xmlns:ns3="12ae8c1a-628e-4358-b6c7-76504a3ed5f5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="232b65a28ae1bbbae5f901744164f207" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2714,6 +2725,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2A8C342-09F0-4130-AE2A-CBE02036160F}">
   <ds:schemaRefs>
@@ -2727,13 +2747,29 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9A7E17E-3835-4720-ADC3-FE5687C9DA33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="56e6d1e7-6899-430c-9877-67183cfe1730"/>
+    <ds:schemaRef ds:uri="12ae8c1a-628e-4358-b6c7-76504a3ed5f5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAC5AF02-6939-4922-8F67-C555D7078AC1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9A7E17E-3835-4720-ADC3-FE5687C9DA33}"/>
 </file>
</xml_diff>